<commit_message>
docs(paper): 四项优化 + final-v1 (16 页)
1. P4 SG 窗口 101→151: 任务数 20→24 (射击8+拍照16), verify ALL PASS
2. EDA 图引入 02_analysis 章节
3. refs.bib 补 5 篇文献 + sections 内引用
4. 02_analysis 填充四问分析 + 数据特征图

xelatex → biber → xelatex × 2 编译通过, 16 页。
</commit_message>
<xml_diff>
--- a/workspace/xupt-2026-b/output/result_v1.xlsx
+++ b/workspace/xupt-2026-b/output/result_v1.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="15.77734375" customWidth="1" min="4" max="4"/>
@@ -709,10 +709,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>454.9</v>
+        <v>449.8</v>
       </c>
       <c r="E10" t="n">
-        <v>455.4</v>
+        <v>450.3</v>
       </c>
     </row>
     <row r="11">
@@ -730,10 +730,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>456.1</v>
+        <v>450.4</v>
       </c>
       <c r="E11" t="n">
-        <v>456.6</v>
+        <v>450.9</v>
       </c>
     </row>
     <row r="12">
@@ -751,10 +751,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>457.1</v>
+        <v>451</v>
       </c>
       <c r="E12" t="n">
-        <v>457.6</v>
+        <v>451.5</v>
       </c>
     </row>
     <row r="13">
@@ -772,10 +772,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>457.9</v>
+        <v>451.6</v>
       </c>
       <c r="E13" t="n">
-        <v>458.4</v>
+        <v>452.1</v>
       </c>
     </row>
     <row r="14">
@@ -793,10 +793,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>458.5</v>
+        <v>453.3</v>
       </c>
       <c r="E14" t="n">
-        <v>459</v>
+        <v>453.8</v>
       </c>
     </row>
     <row r="15">
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>459.4</v>
+        <v>453.9</v>
       </c>
       <c r="E15" t="n">
-        <v>459.9</v>
+        <v>454.4</v>
       </c>
     </row>
     <row r="16">
@@ -826,19 +826,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>S04</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>479.2</v>
+        <v>455.4</v>
       </c>
       <c r="E16" t="n">
-        <v>479.7</v>
+        <v>456.9</v>
       </c>
     </row>
     <row r="17">
@@ -847,19 +847,19 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>P01</t>
+          <t>S03</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>509.8</v>
+        <v>457.8</v>
       </c>
       <c r="E17" t="n">
-        <v>510.3</v>
+        <v>459.3</v>
       </c>
     </row>
     <row r="18">
@@ -868,19 +868,19 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>P02</t>
+          <t>S05</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>510.6</v>
+        <v>459.7</v>
       </c>
       <c r="E18" t="n">
-        <v>511.1</v>
+        <v>461.2</v>
       </c>
     </row>
     <row r="19">
@@ -889,7 +889,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S07</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>809</v>
+        <v>461.3</v>
       </c>
       <c r="E19" t="n">
-        <v>810.5</v>
+        <v>462.8</v>
       </c>
     </row>
     <row r="20">
@@ -910,7 +910,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>810.6</v>
+        <v>491.9</v>
       </c>
       <c r="E20" t="n">
-        <v>812.1</v>
+        <v>493.4</v>
       </c>
     </row>
     <row r="21">
@@ -931,19 +931,103 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>507.2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>508.7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>508.8</v>
+      </c>
+      <c r="E22" t="n">
+        <v>509.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>拍照</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>509.9</v>
+      </c>
+      <c r="E23" t="n">
+        <v>510.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>512.2</v>
+      </c>
+      <c r="E24" t="n">
+        <v>513.7</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>射击</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>812.2</v>
-      </c>
-      <c r="E21" t="n">
-        <v>813.7</v>
+      <c r="D25" t="n">
+        <v>772.1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>773.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>